<commit_message>
- Readme updated, meas_images updated
</commit_message>
<xml_diff>
--- a/beadando/mandelbrot/mandelbrot_opencl_meresek.xlsx
+++ b/beadando/mandelbrot/mandelbrot_opencl_meresek.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xaver\Documents\2025_26_codes\par_dev_programming\c_sdk_220203\par_dev_2026\beadando\mandelbrot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AF795EF-C2E9-4CF4-9EAC-9948FE8428EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E029FA34-3A7F-4815-A463-55288C6EC022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-15" windowWidth="29040" windowHeight="15840" xr2:uid="{0A643644-B1A4-4281-BB52-66989A9493B3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="28">
   <si>
     <t>Mandelbrot-halmaz mérések:</t>
   </si>
@@ -48,9 +48,6 @@
   </si>
   <si>
     <t>Iteráció és felbontás u.a.</t>
-  </si>
-  <si>
-    <t>Futásidő (ms)</t>
   </si>
   <si>
     <t>WorkerGroup mérete</t>
@@ -117,6 +114,12 @@
   </si>
   <si>
     <t xml:space="preserve"> 2560x1280</t>
+  </si>
+  <si>
+    <t>GPU Futásidő (ms)</t>
+  </si>
+  <si>
+    <t>CPU Futásidő (ms)</t>
   </si>
 </sst>
 </file>
@@ -332,7 +335,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Futásidő (ms)</c:v>
+                  <c:v>GPU Futásidő (ms)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -428,6 +431,114 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-A716-4DA8-B209-CE7BF838FA9F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Munka1!$F$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CPU Futásidő (ms)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>Munka1!$B$5:$B$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>512</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Munka1!$F$5:$F$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>697</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8F36-4981-8C15-601560B6FAC2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -933,8 +1044,8 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.13395874514851616"/>
-          <c:y val="2.7816411682892908E-2"/>
+          <c:x val="0.34976626890710827"/>
+          <c:y val="2.5040340049898812E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -988,11 +1099,11 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Munka1!$E$19</c:f>
+              <c:f>Munka1!$E$37</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Futásidő (ms)</c:v>
+                  <c:v>GPU Futásidő (ms)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1009,7 +1120,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>Munka1!$C$20:$C$29</c:f>
+              <c:f>Munka1!$C$38:$C$47</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1048,7 +1159,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Munka1!$E$20:$E$29</c:f>
+              <c:f>Munka1!$E$38:$E$47</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1088,6 +1199,114 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-D1B3-4EA0-8A45-4425FAE952F1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Munka1!$F$37</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CPU Futásidő (ms)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>Munka1!$C$38:$C$47</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>800</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2500</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Munka1!$F$38:$F$47</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>117</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>174</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>320</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>436</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>666</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1016</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1251</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1848</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2467</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3078</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F6C6-4841-9F12-631A96819BBD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1114,7 +1333,7 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>Munka1!$C$19</c15:sqref>
+                          <c15:sqref>Munka1!$C$37</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -1141,7 +1360,7 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>Munka1!$C$20:$C$29</c15:sqref>
+                          <c15:sqref>Munka1!$C$38:$C$47</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -1186,7 +1405,7 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>Munka1!$C$20:$C$29</c15:sqref>
+                          <c15:sqref>Munka1!$C$38:$C$47</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -1559,6 +1778,42 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="hu-HU"/>
+              <a:t>Futásidő (</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="hu-HU" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:effectLst/>
+              </a:rPr>
+              <a:t>Iteráció és a workerGroup u.a.</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="hu-HU" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t> )</a:t>
+            </a:r>
+            <a:endParaRPr lang="hu-HU" b="0"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1600,11 +1855,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Munka1!$E$34</c:f>
+              <c:f>Munka1!$E$64</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Futásidő (ms)</c:v>
+                  <c:v>GPU Futásidő (ms)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1619,9 +1874,66 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="hu-HU"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Munka1!$D$35:$D$44</c:f>
+              <c:f>Munka1!$D$65:$D$74</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -1659,7 +1971,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Munka1!$E$35:$E$44</c:f>
+              <c:f>Munka1!$E$65:$E$74</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1699,6 +2011,170 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-72EC-4968-A74E-6CC3BB7050B4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Munka1!$F$64</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CPU Futásidő (ms)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="hu-HU"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Munka1!$D$65:$D$74</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>512x256</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1024x512</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v> 1536x768</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2048x1024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v> 2560x1280</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v> 3072x1536</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v> 3584x1792</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v> 4096x2048</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v> 4608x2304</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v> 5120x2560</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Munka1!$F$65:$F$74</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>166</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>395</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>706</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1056</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1480</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1984</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2583</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3275</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4044</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-38D7-4754-961A-A1A2BB02921D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1940,6 +2416,37 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="hu-HU"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:extLst>
@@ -1999,6 +2506,42 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="hu-HU"/>
+              <a:t>Futásidő (</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="hu-HU" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                <a:effectLst/>
+              </a:rPr>
+              <a:t>Iteráció és a workerGroup u.a.</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="hu-HU" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t> )</a:t>
+            </a:r>
+            <a:endParaRPr lang="hu-HU" b="0"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2039,11 +2582,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Munka1!$E$34</c:f>
+              <c:f>Munka1!$E$64</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Futásidő (ms)</c:v>
+                  <c:v>GPU Futásidő (ms)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2072,9 +2615,66 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="hu-HU"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Munka1!$D$35:$D$44</c:f>
+              <c:f>Munka1!$D$65:$D$74</c:f>
               <c:strCache>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
@@ -2112,7 +2712,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Munka1!$E$35:$E$44</c:f>
+              <c:f>Munka1!$E$65:$E$74</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2152,7 +2752,186 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-DE64-46D4-AAD6-20304DF84D4C}"/>
+              <c16:uniqueId val="{00000000-16D1-4DBD-97FF-A2E5CF6295E1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Munka1!$F$64</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CPU Futásidő (ms)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="hu-HU"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Munka1!$D$65:$D$74</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>512x256</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1024x512</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v> 1536x768</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2048x1024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v> 2560x1280</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v> 3072x1536</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v> 3584x1792</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v> 4096x2048</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v> 4608x2304</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v> 5120x2560</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Munka1!$F$65:$F$74</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>166</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>395</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>706</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1056</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1480</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1984</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2583</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3275</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4044</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-16D1-4DBD-97FF-A2E5CF6295E1}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2394,6 +3173,37 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="hu-HU"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:extLst>
@@ -2495,8 +3305,8 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.13395874514851616"/>
-          <c:y val="2.7816411682892908E-2"/>
+          <c:x val="0.34976626890710827"/>
+          <c:y val="2.5040340049898812E-2"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -2535,10 +3345,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.17660550243719536"/>
-          <c:y val="0.20038442707086676"/>
-          <c:w val="0.81936257967754034"/>
-          <c:h val="0.46539328899478616"/>
+          <c:x val="0.12022491619240665"/>
+          <c:y val="0.11717250519146614"/>
+          <c:w val="0.87574322392869197"/>
+          <c:h val="0.54860518386570067"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -2549,11 +3359,11 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Munka1!$E$19</c:f>
+              <c:f>Munka1!$E$37</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Futásidő (ms)</c:v>
+                  <c:v>GPU Futásidő (ms)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2582,9 +3392,66 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="hu-HU"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Munka1!$C$20:$C$29</c:f>
+              <c:f>Munka1!$C$38:$C$47</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2623,7 +3490,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Munka1!$E$20:$E$29</c:f>
+              <c:f>Munka1!$E$38:$E$47</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2663,7 +3530,185 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-7427-4D44-8AEE-94F5B8656AEB}"/>
+              <c16:uniqueId val="{00000000-DD25-4113-AB24-0324FFD71173}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Munka1!$F$37</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CPU Futásidő (ms)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="hu-HU"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>Munka1!$C$38:$C$47</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>800</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2500</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Munka1!$F$38:$F$47</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>117</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>174</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>320</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>436</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>666</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1016</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1251</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1848</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2467</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3078</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-DD25-4113-AB24-0324FFD71173}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2690,7 +3735,7 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>Munka1!$C$19</c15:sqref>
+                          <c15:sqref>Munka1!$C$37</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -2719,7 +3764,7 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>Munka1!$C$20:$C$29</c15:sqref>
+                          <c15:sqref>Munka1!$C$38:$C$47</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -2764,7 +3809,7 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>Munka1!$C$20:$C$29</c15:sqref>
+                          <c15:sqref>Munka1!$C$38:$C$47</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -2807,7 +3852,7 @@
                 <c:smooth val="0"/>
                 <c:extLst>
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000001-7427-4D44-8AEE-94F5B8656AEB}"/>
+                    <c16:uniqueId val="{00000002-DD25-4113-AB24-0324FFD71173}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -3207,10 +4252,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.1406413461738007"/>
+          <c:x val="0.11293148258668156"/>
           <c:y val="0.15771455008096233"/>
-          <c:w val="0.83161555492205175"/>
-          <c:h val="0.5175182734358067"/>
+          <c:w val="0.85932541439654997"/>
+          <c:h val="0.60556589966692143"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -3225,7 +4270,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Futásidő (ms)</c:v>
+                  <c:v>GPU Futásidő (ms)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3254,6 +4299,63 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="hu-HU"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
               <c:f>Munka1!$B$5:$B$14</c:f>
@@ -3335,7 +4437,187 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-9FE5-4ACB-B0D2-A97F4FE4290C}"/>
+              <c16:uniqueId val="{00000000-D3AD-4C40-B2DF-0EA3241AEDF1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Munka1!$F$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>CPU Futásidő (ms)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="hu-HU"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>Munka1!$B$5:$B$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>512</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Munka1!$F$5:$F$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>697</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>697</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-D3AD-4C40-B2DF-0EA3241AEDF1}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3479,7 +4761,7 @@
                 <c:smooth val="0"/>
                 <c:extLst>
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000001-9FE5-4ACB-B0D2-A97F4FE4290C}"/>
+                    <c16:uniqueId val="{00000002-D3AD-4C40-B2DF-0EA3241AEDF1}"/>
                   </c:ext>
                 </c:extLst>
               </c15:ser>
@@ -7049,16 +8331,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>605791</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>37148</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>240030</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>126683</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>182880</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>167640</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>120015</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7085,16 +8367,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>607695</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>952</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>226695</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>6667</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>607695</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>49530</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>325755</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7121,16 +8403,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>539115</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>117157</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>474345</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>17145</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>228600</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>952</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>510541</xdr:colOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>29527</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7157,23 +8439,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>340995</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>131445</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>93345</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>20955</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>20955</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>125731</xdr:colOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>29527</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Diagram 4">
+        <xdr:cNvPr id="8" name="Diagram 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{60A95D8A-B39D-44BF-BB7A-FC07EEBEFA18}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6D0E8B8A-A9A3-4610-9C9F-EB996330728B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7195,23 +8477,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>563880</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>563880</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>86678</xdr:rowOff>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>529590</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>73343</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Diagram 5">
+        <xdr:cNvPr id="9" name="Diagram 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35221B25-0FD8-41B4-88C8-BBDB651CD4FA}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{509D205B-1FA9-4525-B7AD-4CF6B2A1BA62}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7233,23 +8515,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>91440</xdr:colOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>280034</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>164782</xdr:rowOff>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>480060</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>162877</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="7" name="Diagram 6">
+        <xdr:cNvPr id="10" name="Diagram 9">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C5E12FF3-5A39-468C-98CA-B790F697170D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9CCEC0F0-9A40-4C76-AD5A-B5FAEEECDBB6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7589,30 +8871,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7689CE3C-8FFB-4855-A87C-76D64013B056}">
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="44.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.6640625" style="2" customWidth="1"/>
     <col min="3" max="3" width="8" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="2"/>
+    <col min="5" max="6" width="18.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>1</v>
@@ -7621,10 +8903,13 @@
         <v>2</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>4</v>
+        <v>26</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5" s="2">
         <v>1</v>
       </c>
@@ -7632,13 +8917,16 @@
         <v>500</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E5" s="2">
         <v>854</v>
       </c>
+      <c r="F5" s="2">
+        <v>697</v>
+      </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B6" s="2">
         <v>2</v>
       </c>
@@ -7646,13 +8934,16 @@
         <v>500</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E6" s="2">
         <v>534</v>
       </c>
+      <c r="F6" s="2">
+        <v>697</v>
+      </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B7" s="2">
         <v>4</v>
       </c>
@@ -7660,13 +8951,16 @@
         <v>500</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E7" s="2">
         <v>392</v>
       </c>
+      <c r="F7" s="2">
+        <v>697</v>
+      </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B8" s="2">
         <v>8</v>
       </c>
@@ -7674,13 +8968,16 @@
         <v>500</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E8" s="2">
         <v>322</v>
       </c>
+      <c r="F8" s="2">
+        <v>697</v>
+      </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B9" s="2">
         <v>16</v>
       </c>
@@ -7688,13 +8985,16 @@
         <v>500</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E9" s="2">
         <v>266</v>
       </c>
+      <c r="F9" s="2">
+        <v>697</v>
+      </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B10" s="2">
         <v>32</v>
       </c>
@@ -7702,13 +9002,16 @@
         <v>500</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E10" s="2">
         <v>258</v>
       </c>
+      <c r="F10" s="2">
+        <v>697</v>
+      </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B11" s="2">
         <v>64</v>
       </c>
@@ -7716,13 +9019,16 @@
         <v>500</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E11" s="2">
         <v>241</v>
       </c>
+      <c r="F11" s="2">
+        <v>697</v>
+      </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B12" s="2">
         <v>128</v>
       </c>
@@ -7730,13 +9036,16 @@
         <v>500</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12" s="2">
         <v>249</v>
       </c>
+      <c r="F12" s="2">
+        <v>697</v>
+      </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B13" s="2">
         <v>256</v>
       </c>
@@ -7744,13 +9053,16 @@
         <v>500</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E13" s="2">
         <v>250</v>
       </c>
+      <c r="F13" s="2">
+        <v>697</v>
+      </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B14" s="2">
         <v>512</v>
       </c>
@@ -7758,328 +9070,397 @@
         <v>500</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E14" s="2">
         <v>262</v>
       </c>
+      <c r="F14" s="2">
+        <v>697</v>
+      </c>
     </row>
-    <row r="18" spans="2:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="B18" s="6" t="s">
+    <row r="36" spans="2:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B36" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B37" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B38" s="2">
+        <v>128</v>
+      </c>
+      <c r="C38" s="2">
+        <v>50</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="E38" s="2">
+        <v>252</v>
+      </c>
+      <c r="F38" s="2">
+        <v>117</v>
+      </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B19" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>4</v>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B39" s="2">
+        <v>128</v>
+      </c>
+      <c r="C39" s="2">
+        <v>100</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E39" s="2">
+        <v>246</v>
+      </c>
+      <c r="F39" s="2">
+        <v>174</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B20" s="2">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B40" s="2">
         <v>128</v>
       </c>
-      <c r="C20" s="2">
-        <v>50</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E20" s="2">
-        <v>252</v>
+      <c r="C40" s="2">
+        <v>200</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E40" s="2">
+        <v>239</v>
+      </c>
+      <c r="F40" s="2">
+        <v>320</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B21" s="2">
+    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B41" s="2">
         <v>128</v>
       </c>
-      <c r="C21" s="2">
-        <v>100</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E21" s="2">
-        <v>246</v>
+      <c r="C41" s="2">
+        <v>300</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E41" s="2">
+        <v>229</v>
+      </c>
+      <c r="F41" s="2">
+        <v>436</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B22" s="2">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B42" s="2">
         <v>128</v>
-      </c>
-      <c r="C22" s="2">
-        <v>200</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E22" s="2">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B23" s="2">
-        <v>128</v>
-      </c>
-      <c r="C23" s="2">
-        <v>300</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E23" s="2">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B24" s="2">
-        <v>128</v>
-      </c>
-      <c r="C24" s="2">
-        <v>500</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E24" s="2">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B25" s="2">
-        <v>128</v>
-      </c>
-      <c r="C25" s="2">
-        <v>800</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E25" s="2">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B26" s="2">
-        <v>128</v>
-      </c>
-      <c r="C26" s="2">
-        <v>1000</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E26" s="2">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B27" s="2">
-        <v>128</v>
-      </c>
-      <c r="C27" s="2">
-        <v>1500</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E27" s="2">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B28" s="2">
-        <v>128</v>
-      </c>
-      <c r="C28" s="2">
-        <v>2000</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E28" s="2">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B29" s="2">
-        <v>128</v>
-      </c>
-      <c r="C29" s="2">
-        <v>2500</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E29" s="2">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="33" spans="2:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="B33" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B34" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B35" s="2">
-        <v>256</v>
-      </c>
-      <c r="C35" s="2">
-        <v>500</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E35" s="2">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B36" s="2">
-        <v>256</v>
-      </c>
-      <c r="C36" s="2">
-        <v>500</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E36" s="2">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="37" spans="2:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B37" s="2">
-        <v>256</v>
-      </c>
-      <c r="C37" s="2">
-        <v>500</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E37" s="2">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B38" s="2">
-        <v>256</v>
-      </c>
-      <c r="C38" s="2">
-        <v>500</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E38" s="2">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="39" spans="2:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B39" s="2">
-        <v>256</v>
-      </c>
-      <c r="C39" s="2">
-        <v>500</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E39" s="2">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="40" spans="2:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B40" s="2">
-        <v>256</v>
-      </c>
-      <c r="C40" s="2">
-        <v>500</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E40" s="2">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="41" spans="2:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B41" s="2">
-        <v>256</v>
-      </c>
-      <c r="C41" s="2">
-        <v>500</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E41" s="2">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="42" spans="2:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B42" s="2">
-        <v>256</v>
       </c>
       <c r="C42" s="2">
         <v>500</v>
       </c>
-      <c r="D42" s="4" t="s">
+      <c r="D42" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E42" s="2">
+        <v>248</v>
+      </c>
+      <c r="F42" s="2">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="43" spans="2:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="2">
+        <v>128</v>
+      </c>
+      <c r="C43" s="2">
+        <v>800</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E43" s="2">
+        <v>290</v>
+      </c>
+      <c r="F43" s="2">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B44" s="2">
+        <v>128</v>
+      </c>
+      <c r="C44" s="2">
+        <v>1000</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E44" s="2">
+        <v>296</v>
+      </c>
+      <c r="F44" s="2">
+        <v>1251</v>
+      </c>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B45" s="2">
+        <v>128</v>
+      </c>
+      <c r="C45" s="2">
+        <v>1500</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E45" s="2">
+        <v>308</v>
+      </c>
+      <c r="F45" s="2">
+        <v>1848</v>
+      </c>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B46" s="2">
+        <v>128</v>
+      </c>
+      <c r="C46" s="2">
+        <v>2000</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E46" s="2">
+        <v>312</v>
+      </c>
+      <c r="F46" s="2">
+        <v>2467</v>
+      </c>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B47" s="2">
+        <v>128</v>
+      </c>
+      <c r="C47" s="2">
+        <v>2500</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E47" s="2">
+        <v>351</v>
+      </c>
+      <c r="F47" s="2">
+        <v>3078</v>
+      </c>
+    </row>
+    <row r="63" spans="2:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B63" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="64" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B64" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F64" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="65" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B65" s="2">
+        <v>256</v>
+      </c>
+      <c r="C65" s="2">
+        <v>500</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E65" s="2">
+        <v>240</v>
+      </c>
+      <c r="F65" s="2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="66" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B66" s="2">
+        <v>256</v>
+      </c>
+      <c r="C66" s="2">
+        <v>500</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E66" s="2">
+        <v>238</v>
+      </c>
+      <c r="F66" s="2">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="67" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B67" s="2">
+        <v>256</v>
+      </c>
+      <c r="C67" s="2">
+        <v>500</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E67" s="2">
+        <v>236</v>
+      </c>
+      <c r="F67" s="2">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="68" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B68" s="2">
+        <v>256</v>
+      </c>
+      <c r="C68" s="2">
+        <v>500</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E68" s="2">
+        <v>257</v>
+      </c>
+      <c r="F68" s="2">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="69" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B69" s="2">
+        <v>256</v>
+      </c>
+      <c r="C69" s="2">
+        <v>500</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E69" s="2">
+        <v>266</v>
+      </c>
+      <c r="F69" s="2">
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="70" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B70" s="2">
+        <v>256</v>
+      </c>
+      <c r="C70" s="2">
+        <v>500</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E70" s="2">
+        <v>287</v>
+      </c>
+      <c r="F70" s="2">
+        <v>1480</v>
+      </c>
+    </row>
+    <row r="71" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B71" s="2">
+        <v>256</v>
+      </c>
+      <c r="C71" s="2">
+        <v>500</v>
+      </c>
+      <c r="D71" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E42" s="2">
+      <c r="E71" s="2">
+        <v>295</v>
+      </c>
+      <c r="F71" s="2">
+        <v>1984</v>
+      </c>
+    </row>
+    <row r="72" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B72" s="2">
+        <v>256</v>
+      </c>
+      <c r="C72" s="2">
+        <v>500</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E72" s="2">
         <v>335</v>
       </c>
+      <c r="F72" s="2">
+        <v>2583</v>
+      </c>
     </row>
-    <row r="43" spans="2:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="2">
+    <row r="73" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B73" s="2">
         <v>256</v>
       </c>
-      <c r="C43" s="2">
+      <c r="C73" s="2">
         <v>500</v>
       </c>
-      <c r="D43" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E43" s="2">
+      <c r="D73" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E73" s="2">
         <v>353</v>
       </c>
+      <c r="F73" s="2">
+        <v>3275</v>
+      </c>
     </row>
-    <row r="44" spans="2:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B44" s="2">
+    <row r="74" spans="2:6" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B74" s="2">
         <v>256</v>
       </c>
-      <c r="C44" s="2">
+      <c r="C74" s="2">
         <v>500</v>
       </c>
-      <c r="D44" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E44" s="2">
+      <c r="D74" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E74" s="2">
         <v>418</v>
+      </c>
+      <c r="F74" s="2">
+        <v>4044</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- readme fix, diagram fix
</commit_message>
<xml_diff>
--- a/beadando/mandelbrot/mandelbrot_opencl_meresek.xlsx
+++ b/beadando/mandelbrot/mandelbrot_opencl_meresek.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xaver\Documents\2025_26_codes\par_dev_programming\c_sdk_220203\par_dev_2026\beadando\mandelbrot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E029FA34-3A7F-4815-A463-55288C6EC022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D84E55C4-C260-45A8-AD3F-C64CA7BF2048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-15" windowWidth="29040" windowHeight="15840" xr2:uid="{0A643644-B1A4-4281-BB52-66989A9493B3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{0A643644-B1A4-4281-BB52-66989A9493B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Munka1" sheetId="1" r:id="rId1"/>
@@ -253,7 +253,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -266,15 +266,15 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" b="1"/>
               <a:t>Futásidő</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="hu-HU"/>
+              <a:rPr lang="hu-HU" b="1"/>
               <a:t> (Iteráció és felbontás u.a.)</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" b="1"/>
               <a:t> </a:t>
             </a:r>
           </a:p>
@@ -293,7 +293,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -316,10 +316,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.1406413461738007"/>
+          <c:x val="0.10970179777845307"/>
           <c:y val="0.15771455008096233"/>
-          <c:w val="0.83161555492205175"/>
-          <c:h val="0.5175182734358067"/>
+          <c:w val="0.86255515080644229"/>
+          <c:h val="0.65829244854488755"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -350,6 +350,64 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="0\ &quot;ms&quot;" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="hu-HU"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
               <c:f>Munka1!$B$5:$B$14</c:f>
@@ -458,6 +516,64 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="0\ &quot;ms&quot;" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="hu-HU"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
               <c:f>Munka1!$B$5:$B$14</c:f>
@@ -701,7 +817,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -714,7 +830,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="hu-HU"/>
+                  <a:rPr lang="hu-HU" sz="1800"/>
                   <a:t>WorkGroup</a:t>
                 </a:r>
               </a:p>
@@ -733,7 +849,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -771,7 +887,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -821,7 +937,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -834,8 +950,8 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="hu-HU"/>
-                  <a:t>Futásidő</a:t>
+                  <a:rPr lang="hu-HU" sz="1800"/>
+                  <a:t>Futásidő (ms)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -853,7 +969,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -885,7 +1001,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1008,7 +1124,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1021,22 +1137,22 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" b="1"/>
               <a:t>Futásidő </a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="hu-HU"/>
+              <a:rPr lang="hu-HU" b="1"/>
               <a:t>(</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" b="1"/>
               <a:t>Felbontás és a workerGroup u.a.</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="hu-HU"/>
+              <a:rPr lang="hu-HU" b="1"/>
               <a:t>)</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="en-US" b="1"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -1061,7 +1177,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -1118,6 +1234,92 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0"/>
+                  <c:y val="-2.8779045591673384E-3"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-A58E-48B3-AA95-D2C81B7FC113}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0"/>
+                  <c:y val="-8.6337136775020158E-3"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-A58E-48B3-AA95-D2C81B7FC113}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:numFmt formatCode="0\ &quot;ms&quot;" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="hu-HU"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
               <c:f>Munka1!$C$38:$C$47</c:f>
@@ -1226,6 +1428,113 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="4.1220115416322912E-3"/>
+                  <c:y val="5.7558091183345711E-3"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-A58E-48B3-AA95-D2C81B7FC113}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="5.4960153888430384E-3"/>
+                  <c:y val="5.7558091183346769E-3"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-A58E-48B3-AA95-D2C81B7FC113}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-5.0379559075429483E-17"/>
+                  <c:y val="-8.6337136775020158E-3"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-A58E-48B3-AA95-D2C81B7FC113}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:numFmt formatCode="0\ &quot;ms&quot;" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="hu-HU"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
               <c:f>Munka1!$C$38:$C$47</c:f>
@@ -1469,7 +1778,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -1482,7 +1791,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="hu-HU"/>
+                  <a:rPr lang="hu-HU" sz="1800"/>
                   <a:t>Iteráció</a:t>
                 </a:r>
               </a:p>
@@ -1509,7 +1818,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -1547,7 +1856,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1597,7 +1906,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -1610,8 +1919,8 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="hu-HU"/>
-                  <a:t>Futásidő</a:t>
+                  <a:rPr lang="hu-HU" sz="1800"/>
+                  <a:t>Futásidő (ms)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -1629,7 +1938,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -1661,7 +1970,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -1690,6 +1999,16 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.37714436561052295"/>
+          <c:y val="0.86153606134884653"/>
+          <c:w val="0.25395529186221877"/>
+          <c:h val="4.5928056887922716E-2"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -1875,6 +2194,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="0\ &quot;ms&quot;" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -2039,6 +2359,7 @@
           </c:spPr>
           <c:invertIfNegative val="0"/>
           <c:dLbls>
+            <c:numFmt formatCode="0\ &quot;ms&quot;" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -2205,7 +2526,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -2218,7 +2539,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="hu-HU"/>
+                  <a:rPr lang="hu-HU" sz="1800"/>
                   <a:t>Felbontás</a:t>
                 </a:r>
               </a:p>
@@ -2237,7 +2558,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -2325,7 +2646,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -2338,8 +2659,8 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="hu-HU"/>
-                  <a:t>Futásidő</a:t>
+                  <a:rPr lang="hu-HU" sz="1800"/>
+                  <a:t>Futásidő (ms)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -2357,7 +2678,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -2573,7 +2894,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="7.6471063880704238E-2"/>
+          <c:y val="9.8258173040418589E-2"/>
+          <c:w val="0.90968906495432966"/>
+          <c:h val="0.72926543197279903"/>
+        </c:manualLayout>
+      </c:layout>
       <c:lineChart>
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
@@ -2616,6 +2947,29 @@
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-4.8031327365697138E-2"/>
+                  <c:y val="2.2498233183115557E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-B76B-4F5F-B37A-E89D89775F1E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:numFmt formatCode="0\ &quot;ms&quot;" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -2645,6 +2999,7 @@
                 <a:endParaRPr lang="hu-HU"/>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="b"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
             <c:showCatName val="0"/>
@@ -2795,6 +3150,29 @@
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-1.8074871741445939E-2"/>
+                  <c:y val="-5.1639238937890748E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-B76B-4F5F-B37A-E89D89775F1E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:numFmt formatCode="0\ &quot;ms&quot;" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -2824,6 +3202,7 @@
                 <a:endParaRPr lang="hu-HU"/>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="t"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
             <c:showCatName val="0"/>
@@ -2833,21 +3212,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
+                <c15:showLeaderLines val="0"/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -2962,7 +3327,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -2975,7 +3340,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="hu-HU"/>
+                  <a:rPr lang="hu-HU" sz="1800"/>
                   <a:t>Felbontás</a:t>
                 </a:r>
               </a:p>
@@ -2994,7 +3359,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -3032,7 +3397,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -3082,7 +3447,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -3095,8 +3460,8 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="hu-HU"/>
-                  <a:t>Futásidő</a:t>
+                  <a:rPr lang="hu-HU" sz="1800"/>
+                  <a:t>Futásidő (ms)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -3114,7 +3479,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -3146,7 +3511,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -3269,7 +3634,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -3282,22 +3647,22 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" b="1"/>
               <a:t>Futásidő </a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="hu-HU"/>
+              <a:rPr lang="hu-HU" b="1"/>
               <a:t>(</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" b="1"/>
               <a:t>Felbontás és a workerGroup u.a.</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="hu-HU"/>
+              <a:rPr lang="hu-HU" b="1"/>
               <a:t>)</a:t>
             </a:r>
-            <a:endParaRPr lang="en-US"/>
+            <a:endParaRPr lang="en-US" b="1"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -3322,7 +3687,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -3345,10 +3710,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.12022491619240665"/>
+          <c:x val="8.9971890889876394E-2"/>
           <c:y val="0.11717250519146614"/>
-          <c:w val="0.87574322392869197"/>
-          <c:h val="0.54860518386570067"/>
+          <c:w val="0.89362001160745996"/>
+          <c:h val="0.69467086849130799"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -3356,7 +3721,7 @@
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="1"/>
-          <c:order val="1"/>
+          <c:order val="0"/>
           <c:tx>
             <c:strRef>
               <c:f>Munka1!$E$37</c:f>
@@ -3393,6 +3758,29 @@
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-3.8971397139713995E-2"/>
+                  <c:y val="3.1253024555320877E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-6B07-4E32-9BE6-83C4954E2805}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:numFmt formatCode="0\ &quot;ms&quot;" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -3422,6 +3810,7 @@
                 <a:endParaRPr lang="hu-HU"/>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="b"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
             <c:showCatName val="0"/>
@@ -3431,21 +3820,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
+                <c15:showLeaderLines val="0"/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -3536,7 +3911,7 @@
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
-          <c:order val="2"/>
+          <c:order val="1"/>
           <c:tx>
             <c:strRef>
               <c:f>Munka1!$F$37</c:f>
@@ -3571,6 +3946,51 @@
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-2.1094609460946118E-2"/>
+                  <c:y val="-5.0288986892808571E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-6B07-4E32-9BE6-83C4954E2805}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-1.2843784378437844E-2"/>
+                  <c:y val="-4.4850140510669233E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-6B07-4E32-9BE6-83C4954E2805}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:numFmt formatCode="0\ &quot;ms&quot;" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -3600,6 +4020,7 @@
                 <a:endParaRPr lang="hu-HU"/>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="t"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
             <c:showCatName val="0"/>
@@ -3609,21 +4030,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
+                <c15:showLeaderLines val="0"/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -3724,141 +4131,7 @@
         <c:smooth val="0"/>
         <c:axId val="1656191023"/>
         <c:axId val="1656197743"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredLineSeries>
-              <c15:ser>
-                <c:idx val="0"/>
-                <c:order val="0"/>
-                <c:tx>
-                  <c:strRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Munka1!$C$37</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:strCache>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>Iteráció</c:v>
-                      </c:pt>
-                    </c:strCache>
-                  </c:strRef>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="28575" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent1"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:cat>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Munka1!$C$38:$C$47</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="10"/>
-                      <c:pt idx="0">
-                        <c:v>50</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>100</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>200</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>300</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>500</c:v>
-                      </c:pt>
-                      <c:pt idx="5">
-                        <c:v>800</c:v>
-                      </c:pt>
-                      <c:pt idx="6">
-                        <c:v>1000</c:v>
-                      </c:pt>
-                      <c:pt idx="7">
-                        <c:v>1500</c:v>
-                      </c:pt>
-                      <c:pt idx="8">
-                        <c:v>2000</c:v>
-                      </c:pt>
-                      <c:pt idx="9">
-                        <c:v>2500</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:cat>
-                <c:val>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Munka1!$C$38:$C$47</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="10"/>
-                      <c:pt idx="0">
-                        <c:v>50</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>100</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>200</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>300</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>500</c:v>
-                      </c:pt>
-                      <c:pt idx="5">
-                        <c:v>800</c:v>
-                      </c:pt>
-                      <c:pt idx="6">
-                        <c:v>1000</c:v>
-                      </c:pt>
-                      <c:pt idx="7">
-                        <c:v>1500</c:v>
-                      </c:pt>
-                      <c:pt idx="8">
-                        <c:v>2000</c:v>
-                      </c:pt>
-                      <c:pt idx="9">
-                        <c:v>2500</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:val>
-                <c:smooth val="0"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000002-DD25-4113-AB24-0324FFD71173}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredLineSeries>
-          </c:ext>
-        </c:extLst>
+        <c:extLst/>
       </c:lineChart>
       <c:catAx>
         <c:axId val="1656191023"/>
@@ -3874,7 +4147,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -3887,7 +4160,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="hu-HU"/>
+                  <a:rPr lang="hu-HU" sz="1800"/>
                   <a:t>Iteráció</a:t>
                 </a:r>
               </a:p>
@@ -3897,8 +4170,8 @@
             <c:manualLayout>
               <c:xMode val="edge"/>
               <c:yMode val="edge"/>
-              <c:x val="0.44893560179977499"/>
-              <c:y val="0.76875002770766332"/>
+              <c:x val="0.47506323466992367"/>
+              <c:y val="0.8726277361543906"/>
             </c:manualLayout>
           </c:layout>
           <c:overlay val="0"/>
@@ -3914,7 +4187,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -3952,7 +4225,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -4002,7 +4275,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -4015,8 +4288,8 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="hu-HU"/>
-                  <a:t>Futásidő</a:t>
+                  <a:rPr lang="hu-HU" sz="1800"/>
+                  <a:t>Futásidő (ms)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -4034,7 +4307,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -4066,7 +4339,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -4095,6 +4368,16 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.38400639276526077"/>
+          <c:y val="0.94063131142549739"/>
+          <c:w val="0.30074398187850282"/>
+          <c:h val="4.1962248191560914E-2"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -4189,7 +4472,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -4202,15 +4485,15 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" b="1"/>
               <a:t>Futásidő</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="hu-HU"/>
+              <a:rPr lang="hu-HU" b="1"/>
               <a:t> (Iteráció és felbontás u.a.)</a:t>
             </a:r>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" b="1"/>
               <a:t> </a:t>
             </a:r>
           </a:p>
@@ -4229,7 +4512,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+            <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -4252,10 +4535,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.11293148258668156"/>
-          <c:y val="0.15771455008096233"/>
-          <c:w val="0.85932541439654997"/>
-          <c:h val="0.60556589966692143"/>
+          <c:x val="9.5010301131713354E-2"/>
+          <c:y val="9.7304611699140869E-2"/>
+          <c:w val="0.87724655752341818"/>
+          <c:h val="0.6659758899365934"/>
         </c:manualLayout>
       </c:layout>
       <c:lineChart>
@@ -4300,6 +4583,7 @@
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:numFmt formatCode="0\ &quot;ms&quot;" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -4308,7 +4592,7 @@
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="t" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
               <a:lstStyle/>
@@ -4329,6 +4613,7 @@
                 <a:endParaRPr lang="hu-HU"/>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="t"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
             <c:showCatName val="0"/>
@@ -4480,6 +4765,7 @@
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:numFmt formatCode="0\ &quot;ms&quot;" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -4509,6 +4795,7 @@
                 <a:endParaRPr lang="hu-HU"/>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="t"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="1"/>
             <c:showCatName val="0"/>
@@ -4783,7 +5070,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -4796,7 +5083,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="hu-HU"/>
+                  <a:rPr lang="hu-HU" sz="1800"/>
                   <a:t>WorkGroup</a:t>
                 </a:r>
               </a:p>
@@ -4815,7 +5102,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -4853,7 +5140,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -4903,7 +5190,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -4916,8 +5203,8 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="hu-HU"/>
-                  <a:t>Futásidő</a:t>
+                  <a:rPr lang="hu-HU" sz="1800"/>
+                  <a:t>Futásidő (ms)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -4935,7 +5222,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -4967,7 +5254,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -8375,8 +8662,8 @@
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>325755</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8442,13 +8729,13 @@
       <xdr:col>22</xdr:col>
       <xdr:colOff>93345</xdr:colOff>
       <xdr:row>63</xdr:row>
-      <xdr:rowOff>20955</xdr:rowOff>
+      <xdr:rowOff>20954</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>37</xdr:col>
       <xdr:colOff>125731</xdr:colOff>
-      <xdr:row>90</xdr:row>
-      <xdr:rowOff>29527</xdr:rowOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>30479</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8480,13 +8767,13 @@
       <xdr:col>22</xdr:col>
       <xdr:colOff>438150</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>28574</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>37</xdr:col>
       <xdr:colOff>529590</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>73343</xdr:rowOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>160019</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>

<commit_message>
- meas image fix
</commit_message>
<xml_diff>
--- a/beadando/mandelbrot/mandelbrot_opencl_meresek.xlsx
+++ b/beadando/mandelbrot/mandelbrot_opencl_meresek.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xaver\Documents\2025_26_codes\par_dev_programming\c_sdk_220203\par_dev_2026\beadando\mandelbrot\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xaver\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D84E55C4-C260-45A8-AD3F-C64CA7BF2048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E86E40B1-A10D-4628-AE4A-E22E92B98C8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{0A643644-B1A4-4281-BB52-66989A9493B3}"/>
   </bookViews>
@@ -2951,8 +2951,8 @@
               <c:idx val="0"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-4.8031327365697138E-2"/>
-                  <c:y val="2.2498233183115557E-2"/>
+                  <c:x val="-3.2318160365580148E-2"/>
+                  <c:y val="-2.6309257099934057E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -2966,6 +2966,28 @@
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000001-B76B-4F5F-B37A-E89D89775F1E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-3.3861919439734121E-2"/>
+                  <c:y val="-2.552962909586385E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-94A6-4E0E-95F1-5A1AD4B1B69B}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -3009,21 +3031,7 @@
             <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
+                <c15:showLeaderLines val="0"/>
               </c:ext>
             </c:extLst>
           </c:dLbls>
@@ -3154,8 +3162,8 @@
               <c:idx val="0"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-1.8074871741445939E-2"/>
-                  <c:y val="-5.1639238937890748E-2"/>
+                  <c:x val="-5.0929652276844983E-2"/>
+                  <c:y val="-9.4872500338456026E-3"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -3169,6 +3177,28 @@
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000000-B76B-4F5F-B37A-E89D89775F1E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-2.6719573267874226E-2"/>
+                  <c:y val="1.6655530371515379E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-94A6-4E0E-95F1-5A1AD4B1B69B}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -3762,8 +3792,8 @@
               <c:idx val="0"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-3.8971397139713995E-2"/>
-                  <c:y val="3.1253024555320877E-2"/>
+                  <c:x val="-3.3646474883708845E-2"/>
+                  <c:y val="-3.0944695881683106E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -3777,6 +3807,50 @@
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000003-6B07-4E32-9BE6-83C4954E2805}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-3.2219440002949851E-2"/>
+                  <c:y val="-3.1116056933795676E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-65F8-4B7D-A127-17450D1B70B3}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-2.2286135050487835E-2"/>
+                  <c:y val="2.8777976699007994E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-65F8-4B7D-A127-17450D1B70B3}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -3950,8 +4024,8 @@
               <c:idx val="0"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-2.1094609460946118E-2"/>
-                  <c:y val="-5.0288986892808571E-2"/>
+                  <c:x val="-5.5151630950345767E-2"/>
+                  <c:y val="2.6941431906360703E-3"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -3969,11 +4043,33 @@
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-5.7406035879178467E-3"/>
+                  <c:y val="1.517375602201161E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-65F8-4B7D-A127-17450D1B70B3}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
               <c:idx val="2"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-1.2843784378437844E-2"/>
-                  <c:y val="-4.4850140510669233E-2"/>
+                  <c:x val="-3.4129450293809059E-2"/>
+                  <c:y val="-3.1028446945168566E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -9159,7 +9255,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7689CE3C-8FFB-4855-A87C-76D64013B056}">
   <dimension ref="A1:F74"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="44.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="39.6640625" style="2" customWidth="1"/>

</xml_diff>